<commit_message>
Update sample data to use the new philanthropy category name
Replace 7 occurrences of "grants_contributions" with "philanthropy" in sample-payloads.ts to align with the updated revenue category.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a1e7a024-8deb-4e05-bb93-350fde674463
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: a84eb250-c960-4a4f-947b-c72e25480388
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/27fdbaf7-67db-442f-83d4-bebcb570d0b5/a1e7a024-8deb-4e05-bb93-350fde674463/1ucI1Ab
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/api-server/qa-output/Standard_Export_Charter_ADA_Grade-Band.xlsx
+++ b/artifacts/api-server/qa-output/Standard_Export_Charter_ADA_Grade-Band.xlsx
@@ -2056,25 +2056,25 @@
       <c r="A11" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B11" s="31" t="str">
+      <c r="B11" s="31">
         <f>SUM(B9:B10)</f>
-        <v>0</v>
-      </c>
-      <c r="C11" s="31" t="str">
+        <v>175000</v>
+      </c>
+      <c r="C11" s="31">
         <f>SUM(C9:C10)</f>
-        <v>0</v>
-      </c>
-      <c r="D11" s="31" t="str">
+        <v>135000</v>
+      </c>
+      <c r="D11" s="31">
         <f>SUM(D9:D10)</f>
-        <v>0</v>
-      </c>
-      <c r="E11" s="31" t="str">
+        <v>95000</v>
+      </c>
+      <c r="E11" s="31">
         <f>SUM(E9:E10)</f>
-        <v>0</v>
-      </c>
-      <c r="F11" s="31" t="str">
+        <v>55000</v>
+      </c>
+      <c r="F11" s="31">
         <f>SUM(F9:F10)</f>
-        <v>0</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>